<commit_message>
Updated Worklog file for progress report 1
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2_ProgressReport1.xlsx
+++ b/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2_ProgressReport1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4f25ae689476683/Desmond_New/Winter2026_DouglasCollege/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4f25ae689476683/Desmond_New/BC-Health-Platform/DocumentsAndReports/worklog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{081EE152-0B2A-4F77-9E31-2A0711B7E302}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E09C5AC7-09ED-4709-ADB6-A0A706653659}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work Log" sheetId="1" r:id="rId1"/>
@@ -316,9 +316,6 @@
     <t>L12-13</t>
   </si>
   <si>
-    <t>Udemy Streamlit ML Deployment - Lessons 12-13: Capstone (Canada unemployment dashboard with forms, tabs, metrics, matplotlib)</t>
-  </si>
-  <si>
     <t>Sprint 1</t>
   </si>
   <si>
@@ -869,6 +866,9 @@
   </si>
   <si>
     <t>Test navigation between all pages; Verify sidebar navigation works; Git commit and push</t>
+  </si>
+  <si>
+    <t>Udemy Streamlit ML Deployment - Lessons 12-13: Capstone (Canada population trend dashboard with forms, tabs, metrics, matplotlib)</t>
   </si>
 </sst>
 </file>
@@ -976,6 +976,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1226,7 +1227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1396,14 +1397,47 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1411,40 +1445,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="16" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1629,10 +1629,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1933,37 +1929,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="83"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="99"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="103"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="94"/>
+      <c r="G3" s="95"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F4" s="17"/>
@@ -2721,7 +2717,7 @@
         <v>92</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>93</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -2729,7 +2725,7 @@
         <v>77</v>
       </c>
       <c r="B39" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C39" s="26" t="s">
         <v>80</v>
@@ -2738,13 +2734,13 @@
         <v>0.33</v>
       </c>
       <c r="E39" s="78" t="s">
+        <v>94</v>
+      </c>
+      <c r="F39" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="F39" s="30" t="s">
+      <c r="G39" s="23" t="s">
         <v>96</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -2752,7 +2748,7 @@
         <v>77</v>
       </c>
       <c r="B40" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C40" s="26" t="s">
         <v>80</v>
@@ -2761,13 +2757,13 @@
         <v>0.33</v>
       </c>
       <c r="E40" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F40" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="G40" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="G40" s="23" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -2775,7 +2771,7 @@
         <v>77</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C41" s="26" t="s">
         <v>80</v>
@@ -2784,13 +2780,13 @@
         <v>0.33</v>
       </c>
       <c r="E41" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F41" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="G41" s="23" t="s">
         <v>100</v>
-      </c>
-      <c r="G41" s="23" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -2798,7 +2794,7 @@
         <v>77</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C42" s="26" t="s">
         <v>80</v>
@@ -2807,13 +2803,13 @@
         <v>0.33</v>
       </c>
       <c r="E42" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F42" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="G42" s="23" t="s">
         <v>102</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -2821,7 +2817,7 @@
         <v>77</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C43" s="26" t="s">
         <v>80</v>
@@ -2830,13 +2826,13 @@
         <v>0.33</v>
       </c>
       <c r="E43" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F43" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="G43" s="23" t="s">
         <v>104</v>
-      </c>
-      <c r="G43" s="23" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -2844,7 +2840,7 @@
         <v>77</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C44" s="26" t="s">
         <v>80</v>
@@ -2853,13 +2849,13 @@
         <v>0.33</v>
       </c>
       <c r="E44" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F44" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="G44" s="23" t="s">
         <v>106</v>
-      </c>
-      <c r="G44" s="23" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -2867,7 +2863,7 @@
         <v>77</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C45" s="26" t="s">
         <v>80</v>
@@ -2876,13 +2872,13 @@
         <v>0.33</v>
       </c>
       <c r="E45" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F45" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="G45" s="23" t="s">
         <v>108</v>
-      </c>
-      <c r="G45" s="23" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2890,7 +2886,7 @@
         <v>77</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C46" s="26" t="s">
         <v>80</v>
@@ -2899,13 +2895,13 @@
         <v>0.33</v>
       </c>
       <c r="E46" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F46" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="G46" s="23" t="s">
         <v>110</v>
-      </c>
-      <c r="G46" s="23" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -2913,7 +2909,7 @@
         <v>77</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C47" s="26" t="s">
         <v>56</v>
@@ -2922,13 +2918,13 @@
         <v>0.17</v>
       </c>
       <c r="E47" s="78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F47" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="G47" s="23" t="s">
         <v>112</v>
-      </c>
-      <c r="G47" s="23" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -2936,7 +2932,7 @@
         <v>77</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C48" s="26" t="s">
         <v>43</v>
@@ -2945,13 +2941,13 @@
         <v>0.25</v>
       </c>
       <c r="E48" s="78" t="s">
+        <v>113</v>
+      </c>
+      <c r="F48" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="F48" s="30" t="s">
+      <c r="G48" s="23" t="s">
         <v>115</v>
-      </c>
-      <c r="G48" s="23" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
@@ -2959,7 +2955,7 @@
         <v>77</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C49" s="26" t="s">
         <v>56</v>
@@ -2968,13 +2964,13 @@
         <v>0.17</v>
       </c>
       <c r="E49" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F49" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="G49" s="23" t="s">
         <v>117</v>
-      </c>
-      <c r="G49" s="23" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -2982,7 +2978,7 @@
         <v>77</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C50" s="26" t="s">
         <v>43</v>
@@ -2991,21 +2987,21 @@
         <v>0.25</v>
       </c>
       <c r="E50" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F50" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="G50" s="23" t="s">
         <v>119</v>
-      </c>
-      <c r="G50" s="23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C51" s="34" t="s">
         <v>74</v>
@@ -3014,21 +3010,21 @@
         <v>0.5</v>
       </c>
       <c r="E51" s="78" t="s">
+        <v>121</v>
+      </c>
+      <c r="F51" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="F51" s="30" t="s">
+      <c r="G51" s="23" t="s">
         <v>123</v>
-      </c>
-      <c r="G51" s="23" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C52" s="34" t="s">
         <v>74</v>
@@ -3037,21 +3033,21 @@
         <v>0.5</v>
       </c>
       <c r="E52" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F52" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="G52" s="23" t="s">
         <v>125</v>
-      </c>
-      <c r="G52" s="23" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C53" s="34" t="s">
         <v>74</v>
@@ -3060,44 +3056,44 @@
         <v>0.5</v>
       </c>
       <c r="E53" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F53" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="G53" s="23" t="s">
         <v>127</v>
-      </c>
-      <c r="G53" s="23" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B54" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C54" s="34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D54" s="36">
         <v>0.75</v>
       </c>
       <c r="E54" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F54" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="G54" s="23" t="s">
         <v>130</v>
-      </c>
-      <c r="G54" s="23" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B55" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C55" s="34" t="s">
         <v>74</v>
@@ -3106,21 +3102,21 @@
         <v>0.5</v>
       </c>
       <c r="E55" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F55" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="G55" s="23" t="s">
         <v>132</v>
-      </c>
-      <c r="G55" s="23" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B56" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C56" s="34" t="s">
         <v>80</v>
@@ -3129,21 +3125,21 @@
         <v>0.33</v>
       </c>
       <c r="E56" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F56" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="G56" s="23" t="s">
         <v>134</v>
-      </c>
-      <c r="G56" s="23" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B57" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C57" s="30" t="s">
         <v>52</v>
@@ -3152,358 +3148,358 @@
         <v>0.1</v>
       </c>
       <c r="E57" s="78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F57" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="G57" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="G57" s="23" t="s">
-        <v>137</v>
-      </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="90" t="s">
+      <c r="A58" s="83" t="s">
+        <v>245</v>
+      </c>
+      <c r="B58" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C58" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="D58" s="83">
+        <v>0.75</v>
+      </c>
+      <c r="E58" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F58" s="83" t="s">
         <v>246</v>
       </c>
-      <c r="B58" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C58" s="90" t="s">
-        <v>129</v>
-      </c>
-      <c r="D58" s="90">
+      <c r="G58" s="84" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" s="83" t="s">
+        <v>245</v>
+      </c>
+      <c r="B59" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C59" s="83" t="s">
+        <v>20</v>
+      </c>
+      <c r="D59" s="83">
+        <v>1</v>
+      </c>
+      <c r="E59" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F59" s="83" t="s">
+        <v>248</v>
+      </c>
+      <c r="G59" s="84" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="83" t="s">
+        <v>245</v>
+      </c>
+      <c r="B60" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C60" s="83" t="s">
+        <v>14</v>
+      </c>
+      <c r="D60" s="83">
+        <v>1.5</v>
+      </c>
+      <c r="E60" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F60" s="83" t="s">
+        <v>250</v>
+      </c>
+      <c r="G60" s="84" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" s="83" t="s">
+        <v>245</v>
+      </c>
+      <c r="B61" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C61" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="D61" s="83">
         <v>0.75</v>
       </c>
-      <c r="E58" s="88" t="s">
+      <c r="E61" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F61" s="83" t="s">
+        <v>252</v>
+      </c>
+      <c r="G61" s="84" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B62" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C62" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="D62" s="83">
+        <v>0.75</v>
+      </c>
+      <c r="E62" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F62" s="83" t="s">
+        <v>255</v>
+      </c>
+      <c r="G62" s="84" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B63" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C63" s="83" t="s">
+        <v>43</v>
+      </c>
+      <c r="D63" s="83">
+        <v>0.25</v>
+      </c>
+      <c r="E63" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F63" s="83" t="s">
+        <v>257</v>
+      </c>
+      <c r="G63" s="84" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B64" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C64" s="83" t="s">
+        <v>74</v>
+      </c>
+      <c r="D64" s="83">
+        <v>0.5</v>
+      </c>
+      <c r="E64" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F64" s="83" t="s">
+        <v>259</v>
+      </c>
+      <c r="G64" s="84" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B65" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C65" s="83" t="s">
+        <v>74</v>
+      </c>
+      <c r="D65" s="83">
+        <v>0.5</v>
+      </c>
+      <c r="E65" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="F65" s="83" t="s">
+        <v>261</v>
+      </c>
+      <c r="G65" s="84" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B66" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C66" s="83" t="s">
+        <v>74</v>
+      </c>
+      <c r="D66" s="83">
+        <v>0.5</v>
+      </c>
+      <c r="E66" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F58" s="90" t="s">
-        <v>247</v>
-      </c>
-      <c r="G58" s="91" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A59" s="90" t="s">
-        <v>246</v>
-      </c>
-      <c r="B59" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C59" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="D59" s="90">
-        <v>1</v>
-      </c>
-      <c r="E59" s="88" t="s">
+      <c r="F66" s="83" t="s">
+        <v>263</v>
+      </c>
+      <c r="G66" s="84" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B67" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C67" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D67" s="83">
+        <v>0.17</v>
+      </c>
+      <c r="E67" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F59" s="90" t="s">
-        <v>249</v>
-      </c>
-      <c r="G59" s="91" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="90" t="s">
-        <v>246</v>
-      </c>
-      <c r="B60" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C60" s="90" t="s">
-        <v>14</v>
-      </c>
-      <c r="D60" s="90">
-        <v>1.5</v>
-      </c>
-      <c r="E60" s="88" t="s">
+      <c r="F67" s="83" t="s">
+        <v>265</v>
+      </c>
+      <c r="G67" s="84" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B68" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C68" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D68" s="83">
+        <v>0.17</v>
+      </c>
+      <c r="E68" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F60" s="90" t="s">
-        <v>251</v>
-      </c>
-      <c r="G60" s="91" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="90" t="s">
-        <v>246</v>
-      </c>
-      <c r="B61" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C61" s="90" t="s">
-        <v>129</v>
-      </c>
-      <c r="D61" s="90">
-        <v>0.75</v>
-      </c>
-      <c r="E61" s="88" t="s">
+      <c r="F68" s="83" t="s">
+        <v>267</v>
+      </c>
+      <c r="G68" s="84" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B69" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C69" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D69" s="83">
+        <v>0.17</v>
+      </c>
+      <c r="E69" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F61" s="90" t="s">
-        <v>253</v>
-      </c>
-      <c r="G61" s="91" t="s">
+      <c r="F69" s="83" t="s">
+        <v>269</v>
+      </c>
+      <c r="G69" s="84" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="83" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B62" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C62" s="90" t="s">
-        <v>129</v>
-      </c>
-      <c r="D62" s="90">
-        <v>0.75</v>
-      </c>
-      <c r="E62" s="88" t="s">
+      <c r="B70" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C70" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D70" s="83">
+        <v>0.17</v>
+      </c>
+      <c r="E70" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F62" s="90" t="s">
-        <v>256</v>
-      </c>
-      <c r="G62" s="91" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A63" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B63" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C63" s="90" t="s">
+      <c r="F70" s="83" t="s">
+        <v>271</v>
+      </c>
+      <c r="G70" s="84" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B71" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C71" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D71" s="83">
+        <v>0.17</v>
+      </c>
+      <c r="E71" s="82" t="s">
+        <v>207</v>
+      </c>
+      <c r="F71" s="83" t="s">
+        <v>273</v>
+      </c>
+      <c r="G71" s="84" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" s="83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B72" s="83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C72" s="83" t="s">
         <v>43</v>
       </c>
-      <c r="D63" s="90">
+      <c r="D72" s="83">
         <v>0.25</v>
       </c>
-      <c r="E63" s="88" t="s">
+      <c r="E72" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="F63" s="90" t="s">
-        <v>258</v>
-      </c>
-      <c r="G63" s="91" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B64" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C64" s="90" t="s">
-        <v>74</v>
-      </c>
-      <c r="D64" s="90">
-        <v>0.5</v>
-      </c>
-      <c r="E64" s="88" t="s">
-        <v>207</v>
-      </c>
-      <c r="F64" s="90" t="s">
-        <v>260</v>
-      </c>
-      <c r="G64" s="91" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B65" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C65" s="90" t="s">
-        <v>74</v>
-      </c>
-      <c r="D65" s="90">
-        <v>0.5</v>
-      </c>
-      <c r="E65" s="88" t="s">
-        <v>207</v>
-      </c>
-      <c r="F65" s="90" t="s">
-        <v>262</v>
-      </c>
-      <c r="G65" s="91" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B66" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C66" s="90" t="s">
-        <v>74</v>
-      </c>
-      <c r="D66" s="90">
-        <v>0.5</v>
-      </c>
-      <c r="E66" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F66" s="90" t="s">
-        <v>264</v>
-      </c>
-      <c r="G66" s="91" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B67" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C67" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="D67" s="90">
-        <v>0.17</v>
-      </c>
-      <c r="E67" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F67" s="90" t="s">
-        <v>266</v>
-      </c>
-      <c r="G67" s="91" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B68" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C68" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="D68" s="90">
-        <v>0.17</v>
-      </c>
-      <c r="E68" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F68" s="90" t="s">
-        <v>268</v>
-      </c>
-      <c r="G68" s="91" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A69" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B69" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C69" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="D69" s="90">
-        <v>0.17</v>
-      </c>
-      <c r="E69" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F69" s="90" t="s">
-        <v>270</v>
-      </c>
-      <c r="G69" s="91" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A70" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B70" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C70" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="D70" s="90">
-        <v>0.17</v>
-      </c>
-      <c r="E70" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F70" s="90" t="s">
-        <v>272</v>
-      </c>
-      <c r="G70" s="91" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A71" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B71" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C71" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="D71" s="90">
-        <v>0.17</v>
-      </c>
-      <c r="E71" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F71" s="90" t="s">
-        <v>274</v>
-      </c>
-      <c r="G71" s="91" t="s">
+      <c r="F72" s="83" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A72" s="90" t="s">
-        <v>255</v>
-      </c>
-      <c r="B72" s="90" t="s">
-        <v>94</v>
-      </c>
-      <c r="C72" s="90" t="s">
-        <v>43</v>
-      </c>
-      <c r="D72" s="90">
-        <v>0.25</v>
-      </c>
-      <c r="E72" s="89" t="s">
-        <v>208</v>
-      </c>
-      <c r="F72" s="90" t="s">
+      <c r="G72" s="84" t="s">
         <v>276</v>
-      </c>
-      <c r="G72" s="91" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
@@ -4182,12 +4178,12 @@
       <c r="G147" s="21"/>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A148" s="92" t="s">
-        <v>138</v>
-      </c>
-      <c r="B148" s="93"/>
-      <c r="C148" s="93"/>
-      <c r="D148" s="94"/>
+      <c r="A148" s="89" t="s">
+        <v>137</v>
+      </c>
+      <c r="B148" s="90"/>
+      <c r="C148" s="90"/>
+      <c r="D148" s="91"/>
       <c r="E148" s="79">
         <f>SUM(D6:D147)</f>
         <v>49.61</v>
@@ -4296,47 +4292,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="102" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+    </row>
+    <row r="3" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="101" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
-    </row>
-    <row r="3" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="86" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
+      <c r="B3" s="97"/>
+      <c r="C3" s="97"/>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="38" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="D4" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="E4" s="38" t="s">
         <v>143</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -4344,7 +4340,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5" s="41">
         <v>5</v>
@@ -4363,7 +4359,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C6" s="41">
         <v>15</v>
@@ -4382,7 +4378,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="47" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C7" s="41">
         <v>25</v>
@@ -4401,7 +4397,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C8" s="41">
         <v>20</v>
@@ -4420,7 +4416,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C9" s="41">
         <v>20</v>
@@ -4439,7 +4435,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C10" s="41">
         <v>15</v>
@@ -4458,23 +4454,23 @@
         <v>6</v>
       </c>
       <c r="B11" s="55" t="s">
-        <v>151</v>
-      </c>
-      <c r="C11" s="97">
+        <v>150</v>
+      </c>
+      <c r="C11" s="86">
         <v>18</v>
       </c>
-      <c r="D11" s="98">
+      <c r="D11" s="87">
         <f>SUM(B63)</f>
         <v>6.5</v>
       </c>
-      <c r="E11" s="99">
+      <c r="E11" s="88">
         <f t="shared" si="0"/>
         <v>0.3611111111111111</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B12" s="57"/>
       <c r="C12" s="58">
@@ -4491,112 +4487,112 @@
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="86" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="81"/>
-      <c r="C14" s="81"/>
-      <c r="D14" s="81"/>
-      <c r="E14" s="81"/>
-      <c r="F14" s="81"/>
-      <c r="G14" s="81"/>
-      <c r="H14" s="81"/>
-      <c r="I14" s="81"/>
-      <c r="J14" s="81"/>
-      <c r="K14" s="81"/>
-      <c r="L14" s="81"/>
-      <c r="M14" s="81"/>
-      <c r="N14" s="81"/>
+      <c r="A14" s="101" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="97"/>
+      <c r="C14" s="97"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="97"/>
+      <c r="G14" s="97"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="97"/>
+      <c r="J14" s="97"/>
+      <c r="K14" s="97"/>
+      <c r="L14" s="97"/>
+      <c r="M14" s="97"/>
+      <c r="N14" s="97"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="C15" s="38" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="D15" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="E15" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="E15" s="38" t="s">
+      <c r="F15" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="F15" s="38" t="s">
+      <c r="G15" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="G15" s="38" t="s">
+      <c r="H15" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="H15" s="38" t="s">
+      <c r="I15" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="I15" s="38" t="s">
+      <c r="J15" s="38" t="s">
         <v>162</v>
       </c>
-      <c r="J15" s="38" t="s">
+      <c r="K15" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="K15" s="38" t="s">
+      <c r="L15" s="38" t="s">
         <v>164</v>
       </c>
-      <c r="L15" s="38" t="s">
+      <c r="M15" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="M15" s="38" t="s">
+      <c r="N15" s="38" t="s">
         <v>166</v>
-      </c>
-      <c r="N15" s="38" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="61"/>
       <c r="B16" s="61" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" s="61" t="s">
         <v>168</v>
       </c>
-      <c r="C16" s="61" t="s">
+      <c r="D16" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="E16" s="61" t="s">
         <v>170</v>
       </c>
-      <c r="E16" s="61" t="s">
+      <c r="F16" s="61" t="s">
         <v>171</v>
       </c>
-      <c r="F16" s="61" t="s">
+      <c r="G16" s="61" t="s">
         <v>172</v>
       </c>
-      <c r="G16" s="61" t="s">
+      <c r="H16" s="61" t="s">
         <v>173</v>
       </c>
-      <c r="H16" s="61" t="s">
+      <c r="I16" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="I16" s="61" t="s">
+      <c r="J16" s="61" t="s">
         <v>175</v>
       </c>
-      <c r="J16" s="61" t="s">
+      <c r="K16" s="61" t="s">
         <v>176</v>
       </c>
-      <c r="K16" s="61" t="s">
+      <c r="L16" s="61" t="s">
         <v>177</v>
       </c>
-      <c r="L16" s="61" t="s">
+      <c r="M16" s="61" t="s">
         <v>178</v>
       </c>
-      <c r="M16" s="61" t="s">
+      <c r="N16" s="61" t="s">
         <v>179</v>
-      </c>
-      <c r="N16" s="61" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="56" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B17" s="62"/>
       <c r="C17" s="40"/>
@@ -4614,7 +4610,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="56" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B18" s="63"/>
       <c r="C18" s="45"/>
@@ -4632,7 +4628,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="65" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B19" s="57"/>
       <c r="C19" s="45"/>
@@ -4650,7 +4646,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="65" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B20" s="57"/>
       <c r="C20" s="45"/>
@@ -4668,7 +4664,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="65" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B21" s="57"/>
       <c r="C21" s="45"/>
@@ -4686,7 +4682,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="65" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B22" s="57"/>
       <c r="C22" s="45"/>
@@ -4704,7 +4700,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="65" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B23" s="57"/>
       <c r="C23" s="57"/>
@@ -4722,7 +4718,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="56" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B24" s="57"/>
       <c r="C24" s="57"/>
@@ -4740,7 +4736,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="65" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B25" s="57"/>
       <c r="C25" s="57"/>
@@ -4758,7 +4754,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="65" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B26" s="57"/>
       <c r="C26" s="57"/>
@@ -4776,7 +4772,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="65" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B27" s="57"/>
       <c r="C27" s="57"/>
@@ -4794,7 +4790,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="65" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B28" s="57"/>
       <c r="C28" s="57"/>
@@ -4812,7 +4808,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="56" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B29" s="57"/>
       <c r="C29" s="57"/>
@@ -4830,7 +4826,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="65" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B30" s="57"/>
       <c r="C30" s="57"/>
@@ -4848,7 +4844,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="65" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B31" s="57"/>
       <c r="C31" s="57"/>
@@ -4866,7 +4862,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="65" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B32" s="57"/>
       <c r="C32" s="57"/>
@@ -4884,7 +4880,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="65" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B33" s="57"/>
       <c r="C33" s="57"/>
@@ -4902,7 +4898,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="56" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B34" s="57"/>
       <c r="C34" s="57"/>
@@ -4920,14 +4916,14 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="65" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B35" s="57"/>
       <c r="C35" s="57"/>
       <c r="D35" s="57"/>
       <c r="E35" s="57"/>
       <c r="F35" s="69" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G35" s="57"/>
       <c r="H35" s="51"/>
@@ -4940,7 +4936,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="65" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B36" s="57"/>
       <c r="C36" s="57"/>
@@ -4955,12 +4951,12 @@
       <c r="L36" s="57"/>
       <c r="M36" s="57"/>
       <c r="N36" s="69" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="56" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B37" s="57"/>
       <c r="C37" s="57"/>
@@ -4978,7 +4974,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="65" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B38" s="57"/>
       <c r="C38" s="57"/>
@@ -4996,7 +4992,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="65" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B39" s="57"/>
       <c r="C39" s="57"/>
@@ -5014,7 +5010,7 @@
     </row>
     <row r="40" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="56" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B40" s="57"/>
       <c r="C40" s="57"/>
@@ -5030,8 +5026,8 @@
       <c r="M40" s="55"/>
       <c r="N40" s="55"/>
     </row>
-    <row r="41" spans="1:14" s="96" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="95"/>
+    <row r="41" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="85"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
@@ -5044,7 +5040,7 @@
     </row>
     <row r="43" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="70" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="4"/>
@@ -5070,7 +5066,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B46" s="42">
         <f>SUMIF('Work Log'!E:E,"1A: UI Mockups",'Work Log'!D:D)</f>
@@ -5080,7 +5076,7 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="45" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B47" s="42">
         <f>SUMIF('Work Log'!E:E,"1B: Project Structure",'Work Log'!D:D)</f>
@@ -5090,7 +5086,7 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="45" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B48" s="42">
         <f>SUMIF('Work Log'!E:E,"1C: Database Setup",'Work Log'!D:D)</f>
@@ -5100,7 +5096,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B49" s="42">
         <f>SUMIF('Work Log'!E:E,"1D: Authentication Feature",'Work Log'!D:D)</f>
@@ -5110,7 +5106,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B50" s="42">
         <f>SUMIF('Work Log'!E:E,"1E: Basic Navigation",'Work Log'!D:D)</f>
@@ -5120,7 +5116,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B51" s="42">
         <f>SUMIF('Work Log'!E:E,"2A: Open AI Integration",'Work Log'!D:D)</f>
@@ -5130,7 +5126,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="47" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B52" s="42">
         <f>SUMIF('Work Log'!E:E,"2B: Safety Layer - CTAS Rules",'Work Log'!D:D)</f>
@@ -5140,7 +5136,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="47" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B53" s="42">
         <f>SUMIF('Work Log'!E:E,"2C: ML Model Training",'Work Log'!D:D)</f>
@@ -5150,7 +5146,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="47" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B54" s="42">
         <f>SUMIF('Work Log'!E:E,"2D: Chatbot UI + Integration",'Work Log'!D:D)</f>
@@ -5160,7 +5156,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="49" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B55" s="42">
         <f>SUMIF('Work Log'!E:E,"3A: Home Dashboard",'Work Log'!D:D)</f>
@@ -5170,7 +5166,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="49" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B56" s="42">
         <f>SUMIF('Work Log'!E:E,"3B: My Dashboard - Personal Analytics",'Work Log'!D:D)</f>
@@ -5180,7 +5176,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="49" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B57" s="42">
         <f>SUMIF('Work Log'!E:E,"3C: Facility Finder",'Work Log'!D:D)</f>
@@ -5190,7 +5186,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="49" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B58" s="42">
         <f>SUMIF('Work Log'!E:E,"3D: Health Education Library",'Work Log'!D:D)</f>
@@ -5200,7 +5196,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B59" s="42">
         <f>SUMIF('Work Log'!E:E,"4A: System Analytics Data",'Work Log'!D:D)</f>
@@ -5210,7 +5206,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B60" s="42">
         <f>SUMIF('Work Log'!E:E,"4B: System Analytics Dashboard",'Work Log'!D:D)</f>
@@ -5220,7 +5216,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="53" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B61" s="42">
         <f>SUMIF('Work Log'!E:E,"5A: Deployment",'Work Log'!D:D)</f>
@@ -5229,7 +5225,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="53" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B62" s="42">
         <f>SUMIF('Work Log'!E:E,"5B: Testing",'Work Log'!D:D)</f>
@@ -5256,7 +5252,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="73" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B65" s="42">
         <f>SUMIF('Work Log'!E:E,"Proof of Concept",'Work Log'!D:D)</f>
@@ -5265,7 +5261,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B66" s="59">
         <f>SUM(B45:B65)</f>
@@ -5294,7 +5290,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -5305,7 +5301,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -5316,122 +5312,122 @@
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B5" s="9">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B6" s="9">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B7" s="9">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B8" s="9">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B9" s="9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B10" s="9">
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B11" s="9">
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B12" s="9">
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B13" s="9">
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B14" s="9">
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B15" s="9">
         <v>3</v>
@@ -5439,68 +5435,68 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B16" s="9">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B17" s="9">
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B18" s="9">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B19" s="9">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B20" s="9">
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B21" s="9">
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -5511,7 +5507,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -5519,21 +5515,21 @@
         <v>17</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="C23" t="s">
         <v>243</v>
-      </c>
-      <c r="C23" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>